<commit_message>
Cleaned up how albums appear in the JSON for consistency
</commit_message>
<xml_diff>
--- a/data/Depeche Mode Songs.xlsx
+++ b/data/Depeche Mode Songs.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/lindanakasone/Documents/GitHub/sound-and-vision/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C13FB078-1786-ED4F-B3BF-CBFBE11FB79F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{954E7000-B2BB-FC4A-9CD8-84C3922F8D00}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1620" yWindow="5840" windowWidth="28040" windowHeight="22780" xr2:uid="{FE581154-A771-454D-BC0C-F4CC813A6F29}"/>
+    <workbookView xWindow="1620" yWindow="4840" windowWidth="28040" windowHeight="22780" xr2:uid="{FE581154-A771-454D-BC0C-F4CC813A6F29}"/>
   </bookViews>
   <sheets>
     <sheet name="Depeche Mode Songs" sheetId="1" r:id="rId1"/>
@@ -691,9 +691,6 @@
     <t>Sounds Of The Universe</t>
   </si>
   <si>
-    <t>Dave Gahan (age 46); Christian Eigner (age 37); Andrew Phillpott</t>
-  </si>
-  <si>
     <t>Martin Gore (age 46-47)</t>
   </si>
   <si>
@@ -863,6 +860,9 @@
   </si>
   <si>
     <t>Dave Gahan (age 60); Peter Gordeno; Christian Eigner; James Ford; Marta Salogni</t>
+  </si>
+  <si>
+    <t>Dave Gahan (age 46); Christian Eigner; Andrew Phillpott</t>
   </si>
 </sst>
 </file>
@@ -4348,7 +4348,7 @@
         <v>2009</v>
       </c>
       <c r="D186" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
     </row>
     <row r="187" spans="1:4" x14ac:dyDescent="0.2">
@@ -4362,7 +4362,7 @@
         <v>2009</v>
       </c>
       <c r="D187" t="s">
-        <v>222</v>
+        <v>279</v>
       </c>
     </row>
     <row r="188" spans="1:4" x14ac:dyDescent="0.2">
@@ -4376,7 +4376,7 @@
         <v>2009</v>
       </c>
       <c r="D188" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
     </row>
     <row r="189" spans="1:4" x14ac:dyDescent="0.2">
@@ -4390,7 +4390,7 @@
         <v>2009</v>
       </c>
       <c r="D189" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
     </row>
     <row r="190" spans="1:4" x14ac:dyDescent="0.2">
@@ -4404,7 +4404,7 @@
         <v>2009</v>
       </c>
       <c r="D190" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
     </row>
     <row r="191" spans="1:4" x14ac:dyDescent="0.2">
@@ -4418,7 +4418,7 @@
         <v>2009</v>
       </c>
       <c r="D191" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
     </row>
     <row r="192" spans="1:4" x14ac:dyDescent="0.2">
@@ -4432,7 +4432,7 @@
         <v>2009</v>
       </c>
       <c r="D192" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
     </row>
     <row r="193" spans="1:4" x14ac:dyDescent="0.2">
@@ -4446,7 +4446,7 @@
         <v>2009</v>
       </c>
       <c r="D193" t="s">
-        <v>222</v>
+        <v>279</v>
       </c>
     </row>
     <row r="194" spans="1:4" x14ac:dyDescent="0.2">
@@ -4460,7 +4460,7 @@
         <v>2009</v>
       </c>
       <c r="D194" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
     </row>
     <row r="195" spans="1:4" x14ac:dyDescent="0.2">
@@ -4474,7 +4474,7 @@
         <v>2009</v>
       </c>
       <c r="D195" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
     </row>
     <row r="196" spans="1:4" x14ac:dyDescent="0.2">
@@ -4488,7 +4488,7 @@
         <v>2009</v>
       </c>
       <c r="D196" t="s">
-        <v>222</v>
+        <v>279</v>
       </c>
     </row>
     <row r="197" spans="1:4" x14ac:dyDescent="0.2">
@@ -4502,7 +4502,7 @@
         <v>2009</v>
       </c>
       <c r="D197" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
     </row>
     <row r="198" spans="1:4" x14ac:dyDescent="0.2">
@@ -4516,7 +4516,7 @@
         <v>2009</v>
       </c>
       <c r="D198" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
     </row>
     <row r="199" spans="1:4" x14ac:dyDescent="0.2">
@@ -4530,7 +4530,7 @@
         <v>2009</v>
       </c>
       <c r="D199" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
     </row>
     <row r="200" spans="1:4" x14ac:dyDescent="0.2">
@@ -4544,7 +4544,7 @@
         <v>2009</v>
       </c>
       <c r="D200" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
     </row>
     <row r="201" spans="1:4" x14ac:dyDescent="0.2">
@@ -4558,7 +4558,7 @@
         <v>2009</v>
       </c>
       <c r="D201" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
     </row>
     <row r="202" spans="1:4" x14ac:dyDescent="0.2">
@@ -4572,7 +4572,7 @@
         <v>2009</v>
       </c>
       <c r="D202" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
     </row>
     <row r="203" spans="1:4" x14ac:dyDescent="0.2">
@@ -4586,595 +4586,595 @@
         <v>2009</v>
       </c>
       <c r="D203" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
     </row>
     <row r="204" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A204" t="s">
+        <v>223</v>
+      </c>
+      <c r="B204" t="s">
         <v>224</v>
-      </c>
-      <c r="B204" t="s">
-        <v>225</v>
       </c>
       <c r="C204">
         <v>2013</v>
       </c>
       <c r="D204" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
     </row>
     <row r="205" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A205" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="B205" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="C205">
         <v>2013</v>
       </c>
       <c r="D205" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
     </row>
     <row r="206" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A206" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
       <c r="B206" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="C206">
         <v>2013</v>
       </c>
       <c r="D206" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
     </row>
     <row r="207" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A207" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
       <c r="B207" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="C207">
         <v>2013</v>
       </c>
       <c r="D207" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
     </row>
     <row r="208" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A208" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="B208" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="C208">
         <v>2013</v>
       </c>
       <c r="D208" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
     </row>
     <row r="209" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A209" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="B209" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="C209">
         <v>2013</v>
       </c>
       <c r="D209" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
     </row>
     <row r="210" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A210" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="B210" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="C210">
         <v>2013</v>
       </c>
       <c r="D210" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
     </row>
     <row r="211" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A211" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="B211" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="C211">
         <v>2013</v>
       </c>
       <c r="D211" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
     </row>
     <row r="212" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A212" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="B212" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="C212">
         <v>2013</v>
       </c>
       <c r="D212" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
     </row>
     <row r="213" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A213" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="B213" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="C213">
         <v>2013</v>
       </c>
       <c r="D213" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
     </row>
     <row r="214" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A214" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
       <c r="B214" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="C214">
         <v>2013</v>
       </c>
       <c r="D214" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
     </row>
     <row r="215" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A215" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
       <c r="B215" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="C215">
         <v>2013</v>
       </c>
       <c r="D215" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
     </row>
     <row r="216" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A216" t="s">
-        <v>237</v>
+        <v>236</v>
       </c>
       <c r="B216" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="C216">
         <v>2013</v>
       </c>
       <c r="D216" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
     </row>
     <row r="217" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A217" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
       <c r="B217" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
       <c r="C217">
         <v>2017</v>
       </c>
       <c r="D217" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
     </row>
     <row r="218" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A218" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
       <c r="B218" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
       <c r="C218">
         <v>2017</v>
       </c>
       <c r="D218" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
     </row>
     <row r="219" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A219" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
       <c r="B219" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
       <c r="C219">
         <v>2017</v>
       </c>
       <c r="D219" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
     </row>
     <row r="220" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A220" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="B220" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
       <c r="C220">
         <v>2017</v>
       </c>
       <c r="D220" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
     </row>
     <row r="221" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A221" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="B221" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
       <c r="C221">
         <v>2017</v>
       </c>
       <c r="D221" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
     </row>
     <row r="222" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A222" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
       <c r="B222" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
       <c r="C222">
         <v>2017</v>
       </c>
       <c r="D222" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
     </row>
     <row r="223" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A223" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
       <c r="B223" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
       <c r="C223">
         <v>2017</v>
       </c>
       <c r="D223" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
     </row>
     <row r="224" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A224" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
       <c r="B224" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
       <c r="C224">
         <v>2017</v>
       </c>
       <c r="D224" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
     </row>
     <row r="225" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A225" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
       <c r="B225" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
       <c r="C225">
         <v>2017</v>
       </c>
       <c r="D225" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
     </row>
     <row r="226" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A226" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="B226" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
       <c r="C226">
         <v>2017</v>
       </c>
       <c r="D226" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
     </row>
     <row r="227" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A227" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="B227" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
       <c r="C227">
         <v>2017</v>
       </c>
       <c r="D227" t="s">
-        <v>261</v>
+        <v>260</v>
       </c>
     </row>
     <row r="228" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A228" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
       <c r="B228" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
       <c r="C228">
         <v>2017</v>
       </c>
       <c r="D228" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
     </row>
     <row r="229" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A229" t="s">
-        <v>252</v>
+        <v>251</v>
       </c>
       <c r="B229" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
       <c r="C229">
         <v>2017</v>
       </c>
       <c r="D229" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
     </row>
     <row r="230" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A230" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
       <c r="B230" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
       <c r="C230">
         <v>2017</v>
       </c>
       <c r="D230" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
     </row>
     <row r="231" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A231" t="s">
-        <v>254</v>
+        <v>253</v>
       </c>
       <c r="B231" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
       <c r="C231">
         <v>2017</v>
       </c>
       <c r="D231" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
     </row>
     <row r="232" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A232" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
       <c r="B232" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
       <c r="C232">
         <v>2017</v>
       </c>
       <c r="D232" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
     </row>
     <row r="233" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A233" t="s">
+        <v>255</v>
+      </c>
+      <c r="B233" t="s">
         <v>256</v>
-      </c>
-      <c r="B233" t="s">
-        <v>257</v>
       </c>
       <c r="C233">
         <v>2017</v>
       </c>
       <c r="D233" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
     </row>
     <row r="234" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A234" t="s">
+        <v>261</v>
+      </c>
+      <c r="B234" t="s">
         <v>262</v>
-      </c>
-      <c r="B234" t="s">
-        <v>263</v>
       </c>
       <c r="C234">
         <v>2023</v>
       </c>
       <c r="D234" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
     </row>
     <row r="235" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A235" t="s">
-        <v>264</v>
+        <v>263</v>
       </c>
       <c r="B235" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
       <c r="C235">
         <v>2023</v>
       </c>
       <c r="D235" t="s">
-        <v>276</v>
+        <v>275</v>
       </c>
     </row>
     <row r="236" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A236" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
       <c r="B236" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
       <c r="C236">
         <v>2023</v>
       </c>
       <c r="D236" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
     </row>
     <row r="237" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A237" t="s">
-        <v>266</v>
+        <v>265</v>
       </c>
       <c r="B237" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
       <c r="C237">
         <v>2023</v>
       </c>
       <c r="D237" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
     </row>
     <row r="238" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A238" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
       <c r="B238" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
       <c r="C238">
         <v>2023</v>
       </c>
       <c r="D238" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
     </row>
     <row r="239" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A239" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="B239" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
       <c r="C239">
         <v>2023</v>
       </c>
       <c r="D239" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
     </row>
     <row r="240" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A240" t="s">
-        <v>269</v>
+        <v>268</v>
       </c>
       <c r="B240" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
       <c r="C240">
         <v>2023</v>
       </c>
       <c r="D240" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
     </row>
     <row r="241" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A241" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
       <c r="B241" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
       <c r="C241">
         <v>2023</v>
       </c>
       <c r="D241" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
     </row>
     <row r="242" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A242" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="B242" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
       <c r="C242">
         <v>2023</v>
       </c>
       <c r="D242" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
     </row>
     <row r="243" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A243" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
       <c r="B243" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
       <c r="C243">
         <v>2023</v>
       </c>
       <c r="D243" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
     </row>
     <row r="244" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A244" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
       <c r="B244" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
       <c r="C244">
         <v>2023</v>
       </c>
       <c r="D244" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
     </row>
     <row r="245" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A245" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="B245" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
       <c r="C245">
         <v>2023</v>
       </c>
       <c r="D245" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
     </row>
   </sheetData>

</xml_diff>